<commit_message>
chore: improved quiz performance, added Question ID, and throttled total quiz output
</commit_message>
<xml_diff>
--- a/quiz/updated-drill-questions/DR1.xlsx
+++ b/quiz/updated-drill-questions/DR1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\firebrigade\wp-content\plugins\techiquiz\quiz\updated-drill-questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D0E74B-C345-4630-A50E-980E2813839E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF426BED-F9A5-4DB0-A4CB-00DBBB03F760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2527" uniqueCount="1631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2527" uniqueCount="1633">
   <si>
     <t>No, because reverse circulation would be required to release the test plug.</t>
   </si>
@@ -4923,6 +4923,12 @@
   </si>
   <si>
     <t>Driller's Day 1 Study Guide Questions</t>
+  </si>
+  <si>
+    <t>Shut-in the well and notify Supervisor</t>
+  </si>
+  <si>
+    <t>Transferring mud between pits is never an acceptable practice;</t>
   </si>
 </sst>
 </file>
@@ -11058,6 +11064,9 @@
       <c r="H162" s="19" t="s">
         <v>1230</v>
       </c>
+      <c r="I162" s="19" t="s">
+        <v>1631</v>
+      </c>
       <c r="J162" s="19" t="s">
         <v>1490</v>
       </c>
@@ -11644,17 +11653,20 @@
       <c r="F179" s="19" t="s">
         <v>550</v>
       </c>
-      <c r="H179" s="19" t="s">
-        <v>2</v>
+      <c r="G179" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H179" s="19" t="b">
+        <v>0</v>
       </c>
       <c r="I179" s="19" t="s">
-        <v>3</v>
+        <v>1632</v>
       </c>
       <c r="J179" s="19" t="s">
         <v>1606</v>
       </c>
       <c r="K179" s="21" t="s">
-        <v>1375</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>